<commit_message>
🦐 update balance xlsx 07-24 10:29
</commit_message>
<xml_diff>
--- a/deepseek/deepseek_balance.xlsx
+++ b/deepseek/deepseek_balance.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="余额记录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +42,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002E7D32"/>
         <bgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001565C0"/>
+        <bgColor rgb="001565C0"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -426,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -910,6 +920,3354 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-22 16:30</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="C29" t="n">
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-22 16:40</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="C30" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-22 16:50</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="C31" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:00</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>7.58</v>
+      </c>
+      <c r="C32" t="n">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:10</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="C33" t="n">
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:20</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="C34" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:30</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="C35" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:40</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="C36" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-22 17:50</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="C37" t="n">
+        <v>-0.46</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:00</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:10</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="C39" t="n">
+        <v>-0.44</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:20</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:30</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="C41" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:40</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="C42" t="n">
+        <v>-1.3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-22 18:50</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:00</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-0.24</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:10</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-0.42</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:20</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-0.24</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:30</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-0.62</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:40</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-22 19:50</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="C49" t="n">
+        <v>-0.24</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:00</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:10</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:20</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:30</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:40</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-22 20:50</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C55" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:00</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:10</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:20</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="C58" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:30</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="C59" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:40</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-22 21:50</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="C61" t="n">
+        <v>-0.11</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:00</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C62" t="n">
+        <v>-0.22</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:10</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:20</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:30</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="C65" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:40</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C66" t="n">
+        <v>-0.43</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-22 22:50</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C67" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:00</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:10</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:20</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:30</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C71" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:40</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C72" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-22 23:50</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:00</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C74" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:10</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C75" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:20</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:30</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C77" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:40</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C78" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-23 00:50</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:00</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:10</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:20</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:30</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:40</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-23 01:50</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:00</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:10</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:20</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:30</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:40</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-23 02:50</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:00</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:10</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:20</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:30</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:40</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-23 03:50</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:00</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:10</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:20</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:30</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C101" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:40</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C102" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-23 04:50</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C103" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:00</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C104" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:10</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:20</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:30</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:40</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-23 05:50</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:00</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:10</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:20</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:30</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:40</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-07-23 06:50</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:00</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:10</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:20</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:30</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:40</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-07-23 07:50</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C121" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:00</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C122" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:10</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:20</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:30</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:40</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-07-23 08:50</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-07-23 09:00</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-07-23 10:10</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>9.83</v>
+      </c>
+      <c r="C129" t="n">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-07-23 10:20</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C130" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-07-23 10:30</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="C131" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-07-23 10:40</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-07-23 10:50</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:00</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>9.41</v>
+      </c>
+      <c r="C134" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:10</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C135" t="n">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:20</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:30</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>9.380000000000001</v>
+      </c>
+      <c r="C137" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:40</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C138" t="n">
+        <v>-0.1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-07-23 11:50</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:00</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:10</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:20</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:30</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:40</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-07-23 12:50</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:00</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:10</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:20</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:30</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:40</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>9.08</v>
+      </c>
+      <c r="C150" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-07-23 13:50</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="C151" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:00</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:10</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="C153" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:20</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>8.81</v>
+      </c>
+      <c r="C154" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:30</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>8.42</v>
+      </c>
+      <c r="C155" t="n">
+        <v>-0.39</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:40</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="C156" t="n">
+        <v>-0.51</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:50</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="C157" t="n">
+        <v>-0.44</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:00</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="C158" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:10</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>7.41</v>
+      </c>
+      <c r="C159" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:20</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>7.27</v>
+      </c>
+      <c r="C160" t="n">
+        <v>-0.14</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:30</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="C161" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:40</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="C162" t="n">
+        <v>-0.23</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:50</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="C163" t="n">
+        <v>-0.29</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:00</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="C164" t="n">
+        <v>-0.16</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:10</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="C165" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:20</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>6.31</v>
+      </c>
+      <c r="C166" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:30</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="C167" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:40</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="C168" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-07-23 16:50</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="C169" t="n">
+        <v>-0.21</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:00</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="C170" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:10</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="C171" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:20</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="C172" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:30</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="C173" t="n">
+        <v>-0.38</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:40</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="C174" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:50</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="C175" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:00</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="C176" t="n">
+        <v>-0.08</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:10</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="C177" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:20</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="C178" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="C179" t="n">
+        <v>-0.79</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="C180" t="n">
+        <v>-0.06</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:50</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="C181" t="n">
+        <v>-1.36</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:00</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C182" t="n">
+        <v>-0.52</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:10</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C183" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:20</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C184" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:30</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C185" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:40</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C186" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-07-23 19:50</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="C187" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:00</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="C188" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:10</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="C189" t="n">
+        <v>-0.54</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:20</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C190" t="n">
+        <v>-0.35</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:30</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C191" t="n">
+        <v>-0.78</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:40</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C192" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-07-23 20:50</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C193" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:00</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C194" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:10</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C195" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:20</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C196" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:30</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C197" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:40</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C198" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-07-23 21:50</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C199" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:00</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C200" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:10</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C201" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:20</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C202" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:30</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C203" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:40</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C204" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-07-23 22:50</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C205" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:00</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C206" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:10</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C207" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:20</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C208" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:30</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C209" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:40</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C210" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-07-23 23:50</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C211" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:00</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C212" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:10</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C213" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:20</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C214" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:30</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C215" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:40</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C216" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-07-24 00:50</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C217" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:00</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C218" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:10</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C219" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:20</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C220" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:30</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C221" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:40</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C222" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-07-24 01:50</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C223" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:00</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C224" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:10</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C225" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:20</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C226" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:30</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C227" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:40</t>
+        </is>
+      </c>
+      <c r="B228" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C228" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-07-24 02:50</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C229" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:00</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C230" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:10</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C231" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:20</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C232" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:30</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C233" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:40</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C234" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-07-24 03:50</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C235" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:00</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C236" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:10</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C237" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:20</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C238" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:30</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C239" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:40</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C240" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-07-24 04:50</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C241" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:00</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C242" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:10</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C243" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:20</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C244" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:30</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C245" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:40</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C246" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-07-24 05:50</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C247" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:00</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C248" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:10</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C249" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:20</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C250" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:30</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C251" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:40</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-07-24 06:50</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C253" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:00</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C254" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:10</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C255" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:20</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C256" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:30</t>
+        </is>
+      </c>
+      <c r="B257" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C257" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:40</t>
+        </is>
+      </c>
+      <c r="B258" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C258" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-07-24 07:50</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C259" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:00</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C260" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:10</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C261" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:20</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C262" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:30</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C263" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:40</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C264" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-07-24 08:50</t>
+        </is>
+      </c>
+      <c r="B265" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C265" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:00</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C266" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:10</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C267" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:20</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C268" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:30</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C269" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:40</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C270" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-07-24 09:50</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>-0.48</v>
+      </c>
+      <c r="C271" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-07-24 10:00</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="C272" t="n">
+        <v>9.99</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-07-24 10:10</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="C273" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-07-24 10:20</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="C274" t="n">
+        <v>-0.41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>起始余额</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>最终余额</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>今日用量</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>充值金额</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>¥1.66</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>¥-0.07</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>¥10.37</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>¥8.64</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>已欠费</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>¥-0.07</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>¥-0.48</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>¥10.31</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>¥9.90</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>已欠费</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>¥-0.48</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>¥8.80</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>¥0.71</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>¥9.99</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>正常</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>